<commit_message>
Migra Práctica 6 al broker MQTT real de la universidad
Se confirmó que mqtt.mecatronica-ibero.mx es accesible desde fuera del
campus (prueba de publicación + round-trip exitosa), por lo que se
re-ejecutaron las 120 pruebas contra el broker real en vez del Mosquitto
local usado como precaución inicial. Resultados consistentes: 93.33%
accuracy, mismos errores en instrucciones metafóricas.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SZseKNVUPy9mTEztLcRPLq
</commit_message>
<xml_diff>
--- a/data/instrumento_supervision_llm_led.xlsx
+++ b/data/instrumento_supervision_llm_led.xlsx
@@ -514,7 +514,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>1.558</v>
+        <v>1.69</v>
       </c>
       <c r="J2" t="n">
         <v>124</v>
@@ -523,7 +523,7 @@
         <v>33</v>
       </c>
       <c r="L2" t="n">
-        <v>44.42</v>
+        <v>33.13</v>
       </c>
     </row>
     <row r="3">
@@ -558,7 +558,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1.567</v>
+        <v>1.336</v>
       </c>
       <c r="J3" t="n">
         <v>126</v>
@@ -567,7 +567,7 @@
         <v>38</v>
       </c>
       <c r="L3" t="n">
-        <v>43.03</v>
+        <v>51.05</v>
       </c>
     </row>
     <row r="4">
@@ -602,7 +602,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>1.566</v>
+        <v>1.35</v>
       </c>
       <c r="J4" t="n">
         <v>125</v>
@@ -611,7 +611,7 @@
         <v>38</v>
       </c>
       <c r="L4" t="n">
-        <v>42.75</v>
+        <v>50.98</v>
       </c>
     </row>
     <row r="5">
@@ -646,7 +646,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>1.577</v>
+        <v>1.316</v>
       </c>
       <c r="J5" t="n">
         <v>128</v>
@@ -655,7 +655,7 @@
         <v>36</v>
       </c>
       <c r="L5" t="n">
-        <v>39.81</v>
+        <v>51.17</v>
       </c>
     </row>
     <row r="6">
@@ -690,7 +690,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1.431</v>
+        <v>1.192</v>
       </c>
       <c r="J6" t="n">
         <v>124</v>
@@ -699,7 +699,7 @@
         <v>29</v>
       </c>
       <c r="L6" t="n">
-        <v>37.94</v>
+        <v>49.98</v>
       </c>
     </row>
     <row r="7">
@@ -734,7 +734,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>1.431</v>
+        <v>1.308</v>
       </c>
       <c r="J7" t="n">
         <v>124</v>
@@ -743,7 +743,7 @@
         <v>33</v>
       </c>
       <c r="L7" t="n">
-        <v>38.32</v>
+        <v>48.11</v>
       </c>
     </row>
     <row r="8">
@@ -778,7 +778,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>1.613</v>
+        <v>1.429</v>
       </c>
       <c r="J8" t="n">
         <v>126</v>
@@ -787,7 +787,7 @@
         <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>42.12</v>
+        <v>50.99</v>
       </c>
     </row>
     <row r="9">
@@ -822,7 +822,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1.34</v>
+        <v>1.19</v>
       </c>
       <c r="J9" t="n">
         <v>129</v>
@@ -831,7 +831,7 @@
         <v>29</v>
       </c>
       <c r="L9" t="n">
-        <v>43.61</v>
+        <v>49.55</v>
       </c>
     </row>
     <row r="10">
@@ -866,7 +866,7 @@
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>1.545</v>
+        <v>1.32</v>
       </c>
       <c r="J10" t="n">
         <v>126</v>
@@ -875,7 +875,7 @@
         <v>36</v>
       </c>
       <c r="L10" t="n">
-        <v>41.37</v>
+        <v>50.94</v>
       </c>
     </row>
     <row r="11">
@@ -910,7 +910,7 @@
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>1.533</v>
+        <v>1.275</v>
       </c>
       <c r="J11" t="n">
         <v>127</v>
@@ -919,7 +919,7 @@
         <v>33</v>
       </c>
       <c r="L11" t="n">
-        <v>38.86</v>
+        <v>51.36</v>
       </c>
     </row>
     <row r="12">
@@ -954,7 +954,7 @@
         <v>1</v>
       </c>
       <c r="I12" t="n">
-        <v>1.511</v>
+        <v>1.261</v>
       </c>
       <c r="J12" t="n">
         <v>124</v>
@@ -963,7 +963,7 @@
         <v>33</v>
       </c>
       <c r="L12" t="n">
-        <v>38.89</v>
+        <v>51.24</v>
       </c>
     </row>
     <row r="13">
@@ -998,7 +998,7 @@
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>1.525</v>
+        <v>1.344</v>
       </c>
       <c r="J13" t="n">
         <v>123</v>
@@ -1007,7 +1007,7 @@
         <v>37</v>
       </c>
       <c r="L13" t="n">
-        <v>38.61</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="14">
@@ -1042,7 +1042,7 @@
         <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>1.426</v>
+        <v>1.247</v>
       </c>
       <c r="J14" t="n">
         <v>126</v>
@@ -1051,7 +1051,7 @@
         <v>33</v>
       </c>
       <c r="L14" t="n">
-        <v>41.83</v>
+        <v>53.07</v>
       </c>
     </row>
     <row r="15">
@@ -1086,7 +1086,7 @@
         <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>1.507</v>
+        <v>1.308</v>
       </c>
       <c r="J15" t="n">
         <v>128</v>
@@ -1095,7 +1095,7 @@
         <v>36</v>
       </c>
       <c r="L15" t="n">
-        <v>43.3</v>
+        <v>50.27</v>
       </c>
     </row>
     <row r="16">
@@ -1130,7 +1130,7 @@
         <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>1.371</v>
+        <v>1.173</v>
       </c>
       <c r="J16" t="n">
         <v>124</v>
@@ -1139,7 +1139,7 @@
         <v>30</v>
       </c>
       <c r="L16" t="n">
-        <v>42.58</v>
+        <v>50.65</v>
       </c>
     </row>
     <row r="17">
@@ -1174,7 +1174,7 @@
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>1.461</v>
+        <v>1.232</v>
       </c>
       <c r="J17" t="n">
         <v>125</v>
@@ -1183,7 +1183,7 @@
         <v>31</v>
       </c>
       <c r="L17" t="n">
-        <v>38.59</v>
+        <v>50.31</v>
       </c>
     </row>
     <row r="18">
@@ -1218,7 +1218,7 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>1.454</v>
+        <v>1.285</v>
       </c>
       <c r="J18" t="n">
         <v>126</v>
@@ -1227,7 +1227,7 @@
         <v>33</v>
       </c>
       <c r="L18" t="n">
-        <v>38.63</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="19">
@@ -1262,7 +1262,7 @@
         <v>1</v>
       </c>
       <c r="I19" t="n">
-        <v>1.495</v>
+        <v>1.342</v>
       </c>
       <c r="J19" t="n">
         <v>128</v>
@@ -1271,7 +1271,7 @@
         <v>36</v>
       </c>
       <c r="L19" t="n">
-        <v>41.28</v>
+        <v>50.49</v>
       </c>
     </row>
     <row r="20">
@@ -1306,7 +1306,7 @@
         <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>1.314</v>
+        <v>1.165</v>
       </c>
       <c r="J20" t="n">
         <v>127</v>
@@ -1315,7 +1315,7 @@
         <v>29</v>
       </c>
       <c r="L20" t="n">
-        <v>44.95</v>
+        <v>51.44</v>
       </c>
     </row>
     <row r="21">
@@ -1350,7 +1350,7 @@
         <v>1</v>
       </c>
       <c r="I21" t="n">
-        <v>1.468</v>
+        <v>1.255</v>
       </c>
       <c r="J21" t="n">
         <v>127</v>
@@ -1359,7 +1359,7 @@
         <v>33</v>
       </c>
       <c r="L21" t="n">
-        <v>41.75</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="22">
@@ -1394,7 +1394,7 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>1.6</v>
+        <v>1.328</v>
       </c>
       <c r="J22" t="n">
         <v>125</v>
@@ -1403,7 +1403,7 @@
         <v>35</v>
       </c>
       <c r="L22" t="n">
-        <v>38.12</v>
+        <v>48.27</v>
       </c>
     </row>
     <row r="23">
@@ -1438,7 +1438,7 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>1.54</v>
+        <v>1.295</v>
       </c>
       <c r="J23" t="n">
         <v>126</v>
@@ -1447,7 +1447,7 @@
         <v>34</v>
       </c>
       <c r="L23" t="n">
-        <v>38.8</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="24">
@@ -1482,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>1.49</v>
+        <v>1.377</v>
       </c>
       <c r="J24" t="n">
         <v>127</v>
@@ -1491,7 +1491,7 @@
         <v>35</v>
       </c>
       <c r="L24" t="n">
-        <v>37.84</v>
+        <v>47.08</v>
       </c>
     </row>
     <row r="25">
@@ -1526,7 +1526,7 @@
         <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>1.494</v>
+        <v>1.36</v>
       </c>
       <c r="J25" t="n">
         <v>127</v>
@@ -1535,7 +1535,7 @@
         <v>35</v>
       </c>
       <c r="L25" t="n">
-        <v>41.02</v>
+        <v>48.93</v>
       </c>
     </row>
     <row r="26">
@@ -1570,7 +1570,7 @@
         <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>1.323</v>
+        <v>1.235</v>
       </c>
       <c r="J26" t="n">
         <v>126</v>
@@ -1579,7 +1579,7 @@
         <v>29</v>
       </c>
       <c r="L26" t="n">
-        <v>44.56</v>
+        <v>49.49</v>
       </c>
     </row>
     <row r="27">
@@ -1614,7 +1614,7 @@
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>1.625</v>
+        <v>1.37</v>
       </c>
       <c r="J27" t="n">
         <v>127</v>
@@ -1623,7 +1623,7 @@
         <v>36</v>
       </c>
       <c r="L27" t="n">
-        <v>38.81</v>
+        <v>49.04</v>
       </c>
     </row>
     <row r="28">
@@ -1658,7 +1658,7 @@
         <v>1</v>
       </c>
       <c r="I28" t="n">
-        <v>1.611</v>
+        <v>1.388</v>
       </c>
       <c r="J28" t="n">
         <v>129</v>
@@ -1667,7 +1667,7 @@
         <v>37</v>
       </c>
       <c r="L28" t="n">
-        <v>39.42</v>
+        <v>49.13</v>
       </c>
     </row>
     <row r="29">
@@ -1702,7 +1702,7 @@
         <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>1.283</v>
+        <v>1.315</v>
       </c>
       <c r="J29" t="n">
         <v>128</v>
@@ -1711,7 +1711,7 @@
         <v>34</v>
       </c>
       <c r="L29" t="n">
-        <v>48.55</v>
+        <v>48.96</v>
       </c>
     </row>
     <row r="30">
@@ -1746,7 +1746,7 @@
         <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>1.431</v>
+        <v>1.461</v>
       </c>
       <c r="J30" t="n">
         <v>127</v>
@@ -1790,7 +1790,7 @@
         <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>1.28</v>
+        <v>1.314</v>
       </c>
       <c r="J31" t="n">
         <v>127</v>
@@ -1799,7 +1799,7 @@
         <v>35</v>
       </c>
       <c r="L31" t="n">
-        <v>48.97</v>
+        <v>49.23</v>
       </c>
     </row>
     <row r="32">
@@ -1834,7 +1834,7 @@
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>1.217</v>
+        <v>1.279</v>
       </c>
       <c r="J32" t="n">
         <v>124</v>
@@ -1843,7 +1843,7 @@
         <v>33</v>
       </c>
       <c r="L32" t="n">
-        <v>50.38</v>
+        <v>50.58</v>
       </c>
     </row>
     <row r="33">
@@ -1878,7 +1878,7 @@
         <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>1.323</v>
+        <v>1.373</v>
       </c>
       <c r="J33" t="n">
         <v>126</v>
@@ -1887,7 +1887,7 @@
         <v>38</v>
       </c>
       <c r="L33" t="n">
-        <v>50.15</v>
+        <v>50.53</v>
       </c>
     </row>
     <row r="34">
@@ -1922,7 +1922,7 @@
         <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>1.316</v>
+        <v>1.366</v>
       </c>
       <c r="J34" t="n">
         <v>125</v>
@@ -1931,7 +1931,7 @@
         <v>38</v>
       </c>
       <c r="L34" t="n">
-        <v>50.37</v>
+        <v>50.34</v>
       </c>
     </row>
     <row r="35">
@@ -1966,7 +1966,7 @@
         <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>1.277</v>
+        <v>1.324</v>
       </c>
       <c r="J35" t="n">
         <v>128</v>
@@ -1975,7 +1975,7 @@
         <v>36</v>
       </c>
       <c r="L35" t="n">
-        <v>50.52</v>
+        <v>50.22</v>
       </c>
     </row>
     <row r="36">
@@ -2010,7 +2010,7 @@
         <v>1</v>
       </c>
       <c r="I36" t="n">
-        <v>1.157</v>
+        <v>1.199</v>
       </c>
       <c r="J36" t="n">
         <v>124</v>
@@ -2019,7 +2019,7 @@
         <v>29</v>
       </c>
       <c r="L36" t="n">
-        <v>49.22</v>
+        <v>48.97</v>
       </c>
     </row>
     <row r="37">
@@ -2054,7 +2054,7 @@
         <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>1.223</v>
+        <v>1.294</v>
       </c>
       <c r="J37" t="n">
         <v>124</v>
@@ -2063,7 +2063,7 @@
         <v>33</v>
       </c>
       <c r="L37" t="n">
-        <v>49.61</v>
+        <v>49.24</v>
       </c>
     </row>
     <row r="38">
@@ -2098,7 +2098,7 @@
         <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>1.359</v>
+        <v>1.41</v>
       </c>
       <c r="J38" t="n">
         <v>126</v>
@@ -2107,7 +2107,7 @@
         <v>40</v>
       </c>
       <c r="L38" t="n">
-        <v>50.04</v>
+        <v>50.16</v>
       </c>
     </row>
     <row r="39">
@@ -2142,7 +2142,7 @@
         <v>1</v>
       </c>
       <c r="I39" t="n">
-        <v>1.151</v>
+        <v>1.206</v>
       </c>
       <c r="J39" t="n">
         <v>129</v>
@@ -2151,7 +2151,7 @@
         <v>29</v>
       </c>
       <c r="L39" t="n">
-        <v>49.28</v>
+        <v>49.29</v>
       </c>
     </row>
     <row r="40">
@@ -2186,7 +2186,7 @@
         <v>1</v>
       </c>
       <c r="I40" t="n">
-        <v>1.279</v>
+        <v>1.341</v>
       </c>
       <c r="J40" t="n">
         <v>126</v>
@@ -2195,7 +2195,7 @@
         <v>36</v>
       </c>
       <c r="L40" t="n">
-        <v>50.31</v>
+        <v>50.85</v>
       </c>
     </row>
     <row r="41">
@@ -2230,7 +2230,7 @@
         <v>1</v>
       </c>
       <c r="I41" t="n">
-        <v>1.219</v>
+        <v>1.253</v>
       </c>
       <c r="J41" t="n">
         <v>127</v>
@@ -2239,7 +2239,7 @@
         <v>33</v>
       </c>
       <c r="L41" t="n">
-        <v>50.5</v>
+        <v>50.45</v>
       </c>
     </row>
     <row r="42">
@@ -2274,7 +2274,7 @@
         <v>1</v>
       </c>
       <c r="I42" t="n">
-        <v>1.209</v>
+        <v>1.264</v>
       </c>
       <c r="J42" t="n">
         <v>124</v>
@@ -2283,7 +2283,7 @@
         <v>33</v>
       </c>
       <c r="L42" t="n">
-        <v>50.72</v>
+        <v>50.27</v>
       </c>
     </row>
     <row r="43">
@@ -2318,7 +2318,7 @@
         <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>1.297</v>
+        <v>1.346</v>
       </c>
       <c r="J43" t="n">
         <v>123</v>
@@ -2327,7 +2327,7 @@
         <v>37</v>
       </c>
       <c r="L43" t="n">
-        <v>50.15</v>
+        <v>50.76</v>
       </c>
     </row>
     <row r="44">
@@ -2362,7 +2362,7 @@
         <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>1.216</v>
+        <v>1.273</v>
       </c>
       <c r="J44" t="n">
         <v>126</v>
@@ -2371,7 +2371,7 @@
         <v>33</v>
       </c>
       <c r="L44" t="n">
-        <v>50.55</v>
+        <v>50.31</v>
       </c>
     </row>
     <row r="45">
@@ -2406,7 +2406,7 @@
         <v>1</v>
       </c>
       <c r="I45" t="n">
-        <v>1.277</v>
+        <v>1.336</v>
       </c>
       <c r="J45" t="n">
         <v>128</v>
@@ -2415,7 +2415,7 @@
         <v>36</v>
       </c>
       <c r="L45" t="n">
-        <v>50.36</v>
+        <v>50.23</v>
       </c>
     </row>
     <row r="46">
@@ -2450,7 +2450,7 @@
         <v>1</v>
       </c>
       <c r="I46" t="n">
-        <v>1.143</v>
+        <v>1.196</v>
       </c>
       <c r="J46" t="n">
         <v>124</v>
@@ -2459,7 +2459,7 @@
         <v>30</v>
       </c>
       <c r="L46" t="n">
-        <v>51.15</v>
+        <v>50.7</v>
       </c>
     </row>
     <row r="47">
@@ -2494,7 +2494,7 @@
         <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>1.171</v>
+        <v>1.222</v>
       </c>
       <c r="J47" t="n">
         <v>125</v>
@@ -2503,7 +2503,7 @@
         <v>31</v>
       </c>
       <c r="L47" t="n">
-        <v>50.68</v>
+        <v>50.36</v>
       </c>
     </row>
     <row r="48">
@@ -2538,7 +2538,7 @@
         <v>1</v>
       </c>
       <c r="I48" t="n">
-        <v>1.217</v>
+        <v>1.263</v>
       </c>
       <c r="J48" t="n">
         <v>126</v>
@@ -2547,7 +2547,7 @@
         <v>33</v>
       </c>
       <c r="L48" t="n">
-        <v>50.45</v>
+        <v>50.82</v>
       </c>
     </row>
     <row r="49">
@@ -2582,7 +2582,7 @@
         <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>1.29</v>
+        <v>1.32</v>
       </c>
       <c r="J49" t="n">
         <v>128</v>
@@ -2591,7 +2591,7 @@
         <v>36</v>
       </c>
       <c r="L49" t="n">
-        <v>50.22</v>
+        <v>51.63</v>
       </c>
     </row>
     <row r="50">
@@ -2626,7 +2626,7 @@
         <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>1.133</v>
+        <v>1.175</v>
       </c>
       <c r="J50" t="n">
         <v>127</v>
@@ -2635,7 +2635,7 @@
         <v>29</v>
       </c>
       <c r="L50" t="n">
-        <v>50.75</v>
+        <v>50.65</v>
       </c>
     </row>
     <row r="51">
@@ -2670,7 +2670,7 @@
         <v>1</v>
       </c>
       <c r="I51" t="n">
-        <v>1.215</v>
+        <v>1.278</v>
       </c>
       <c r="J51" t="n">
         <v>127</v>
@@ -2679,7 +2679,7 @@
         <v>33</v>
       </c>
       <c r="L51" t="n">
-        <v>50.57</v>
+        <v>50.46</v>
       </c>
     </row>
     <row r="52">
@@ -2714,7 +2714,7 @@
         <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>1.28</v>
+        <v>1.333</v>
       </c>
       <c r="J52" t="n">
         <v>125</v>
@@ -2723,7 +2723,7 @@
         <v>35</v>
       </c>
       <c r="L52" t="n">
-        <v>49.3</v>
+        <v>49.03</v>
       </c>
     </row>
     <row r="53">
@@ -2758,7 +2758,7 @@
         <v>1</v>
       </c>
       <c r="I53" t="n">
-        <v>1.237</v>
+        <v>1.288</v>
       </c>
       <c r="J53" t="n">
         <v>126</v>
@@ -2767,7 +2767,7 @@
         <v>34</v>
       </c>
       <c r="L53" t="n">
-        <v>50.12</v>
+        <v>50.62</v>
       </c>
     </row>
     <row r="54">
@@ -2802,7 +2802,7 @@
         <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>1.28</v>
+        <v>1.325</v>
       </c>
       <c r="J54" t="n">
         <v>127</v>
@@ -2811,7 +2811,7 @@
         <v>35</v>
       </c>
       <c r="L54" t="n">
-        <v>49.12</v>
+        <v>49.18</v>
       </c>
     </row>
     <row r="55">
@@ -2846,7 +2846,7 @@
         <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>1.274</v>
+        <v>1.335</v>
       </c>
       <c r="J55" t="n">
         <v>127</v>
@@ -2855,7 +2855,7 @@
         <v>35</v>
       </c>
       <c r="L55" t="n">
-        <v>48.92</v>
+        <v>48.91</v>
       </c>
     </row>
     <row r="56">
@@ -2890,7 +2890,7 @@
         <v>1</v>
       </c>
       <c r="I56" t="n">
-        <v>1.148</v>
+        <v>1.234</v>
       </c>
       <c r="J56" t="n">
         <v>126</v>
@@ -2899,7 +2899,7 @@
         <v>29</v>
       </c>
       <c r="L56" t="n">
-        <v>50.85</v>
+        <v>49.33</v>
       </c>
     </row>
     <row r="57">
@@ -2934,7 +2934,7 @@
         <v>1</v>
       </c>
       <c r="I57" t="n">
-        <v>1.298</v>
+        <v>1.353</v>
       </c>
       <c r="J57" t="n">
         <v>127</v>
@@ -2943,7 +2943,7 @@
         <v>36</v>
       </c>
       <c r="L57" t="n">
-        <v>49.15</v>
+        <v>49.37</v>
       </c>
     </row>
     <row r="58">
@@ -2978,7 +2978,7 @@
         <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>1.315</v>
+        <v>1.375</v>
       </c>
       <c r="J58" t="n">
         <v>129</v>
@@ -2987,7 +2987,7 @@
         <v>37</v>
       </c>
       <c r="L58" t="n">
-        <v>49.1</v>
+        <v>49.04</v>
       </c>
     </row>
     <row r="59">
@@ -3022,7 +3022,7 @@
         <v>1</v>
       </c>
       <c r="I59" t="n">
-        <v>1.259</v>
+        <v>1.321</v>
       </c>
       <c r="J59" t="n">
         <v>128</v>
@@ -3031,7 +3031,7 @@
         <v>34</v>
       </c>
       <c r="L59" t="n">
-        <v>49.13</v>
+        <v>49.17</v>
       </c>
     </row>
     <row r="60">
@@ -3066,7 +3066,7 @@
         <v>1</v>
       </c>
       <c r="I60" t="n">
-        <v>1.403</v>
+        <v>1.452</v>
       </c>
       <c r="J60" t="n">
         <v>127</v>
@@ -3075,7 +3075,7 @@
         <v>41</v>
       </c>
       <c r="L60" t="n">
-        <v>48.72</v>
+        <v>49.31</v>
       </c>
     </row>
     <row r="61">
@@ -3110,7 +3110,7 @@
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>1.283</v>
+        <v>1.345</v>
       </c>
       <c r="J61" t="n">
         <v>127</v>
@@ -3119,7 +3119,7 @@
         <v>35</v>
       </c>
       <c r="L61" t="n">
-        <v>48.66</v>
+        <v>48.94</v>
       </c>
     </row>
     <row r="62">
@@ -3154,7 +3154,7 @@
         <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>1.214</v>
+        <v>1.27</v>
       </c>
       <c r="J62" t="n">
         <v>124</v>
@@ -3163,7 +3163,7 @@
         <v>33</v>
       </c>
       <c r="L62" t="n">
-        <v>50.35</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="63">
@@ -3198,7 +3198,7 @@
         <v>1</v>
       </c>
       <c r="I63" t="n">
-        <v>1.334</v>
+        <v>1.362</v>
       </c>
       <c r="J63" t="n">
         <v>126</v>
@@ -3207,7 +3207,7 @@
         <v>38</v>
       </c>
       <c r="L63" t="n">
-        <v>50.1</v>
+        <v>50.06</v>
       </c>
     </row>
     <row r="64">
@@ -3242,7 +3242,7 @@
         <v>1</v>
       </c>
       <c r="I64" t="n">
-        <v>1.326</v>
+        <v>1.365</v>
       </c>
       <c r="J64" t="n">
         <v>125</v>
@@ -3251,7 +3251,7 @@
         <v>38</v>
       </c>
       <c r="L64" t="n">
-        <v>50.24</v>
+        <v>50.6</v>
       </c>
     </row>
     <row r="65">
@@ -3286,7 +3286,7 @@
         <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>1.279</v>
+        <v>1.328</v>
       </c>
       <c r="J65" t="n">
         <v>128</v>
@@ -3295,7 +3295,7 @@
         <v>36</v>
       </c>
       <c r="L65" t="n">
-        <v>50.46</v>
+        <v>50.26</v>
       </c>
     </row>
     <row r="66">
@@ -3330,7 +3330,7 @@
         <v>1</v>
       </c>
       <c r="I66" t="n">
-        <v>1.151</v>
+        <v>1.181</v>
       </c>
       <c r="J66" t="n">
         <v>124</v>
@@ -3339,7 +3339,7 @@
         <v>29</v>
       </c>
       <c r="L66" t="n">
-        <v>49.49</v>
+        <v>49.17</v>
       </c>
     </row>
     <row r="67">
@@ -3374,7 +3374,7 @@
         <v>1</v>
       </c>
       <c r="I67" t="n">
-        <v>1.242</v>
+        <v>1.278</v>
       </c>
       <c r="J67" t="n">
         <v>124</v>
@@ -3383,7 +3383,7 @@
         <v>33</v>
       </c>
       <c r="L67" t="n">
-        <v>49.38</v>
+        <v>49.62</v>
       </c>
     </row>
     <row r="68">
@@ -3418,7 +3418,7 @@
         <v>1</v>
       </c>
       <c r="I68" t="n">
-        <v>1.376</v>
+        <v>1.429</v>
       </c>
       <c r="J68" t="n">
         <v>126</v>
@@ -3427,7 +3427,7 @@
         <v>40</v>
       </c>
       <c r="L68" t="n">
-        <v>50.3</v>
+        <v>49.97</v>
       </c>
     </row>
     <row r="69">
@@ -3462,7 +3462,7 @@
         <v>1</v>
       </c>
       <c r="I69" t="n">
-        <v>1.158</v>
+        <v>1.214</v>
       </c>
       <c r="J69" t="n">
         <v>129</v>
@@ -3471,7 +3471,7 @@
         <v>29</v>
       </c>
       <c r="L69" t="n">
-        <v>49.28</v>
+        <v>49.33</v>
       </c>
     </row>
     <row r="70">
@@ -3506,7 +3506,7 @@
         <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>1.281</v>
+        <v>1.327</v>
       </c>
       <c r="J70" t="n">
         <v>126</v>
@@ -3515,7 +3515,7 @@
         <v>36</v>
       </c>
       <c r="L70" t="n">
-        <v>50.76</v>
+        <v>50.37</v>
       </c>
     </row>
     <row r="71">
@@ -3550,7 +3550,7 @@
         <v>1</v>
       </c>
       <c r="I71" t="n">
-        <v>1.223</v>
+        <v>1.261</v>
       </c>
       <c r="J71" t="n">
         <v>127</v>
@@ -3559,7 +3559,7 @@
         <v>33</v>
       </c>
       <c r="L71" t="n">
-        <v>50.78</v>
+        <v>50.73</v>
       </c>
     </row>
     <row r="72">
@@ -3594,7 +3594,7 @@
         <v>1</v>
       </c>
       <c r="I72" t="n">
-        <v>1.967</v>
+        <v>1.269</v>
       </c>
       <c r="J72" t="n">
         <v>124</v>
@@ -3603,7 +3603,7 @@
         <v>33</v>
       </c>
       <c r="L72" t="n">
-        <v>24.28</v>
+        <v>50.69</v>
       </c>
     </row>
     <row r="73">
@@ -3638,7 +3638,7 @@
         <v>1</v>
       </c>
       <c r="I73" t="n">
-        <v>1.31</v>
+        <v>1.352</v>
       </c>
       <c r="J73" t="n">
         <v>123</v>
@@ -3647,7 +3647,7 @@
         <v>37</v>
       </c>
       <c r="L73" t="n">
-        <v>51.1</v>
+        <v>50.32</v>
       </c>
     </row>
     <row r="74">
@@ -3682,7 +3682,7 @@
         <v>1</v>
       </c>
       <c r="I74" t="n">
-        <v>1.22</v>
+        <v>1.273</v>
       </c>
       <c r="J74" t="n">
         <v>126</v>
@@ -3691,7 +3691,7 @@
         <v>33</v>
       </c>
       <c r="L74" t="n">
-        <v>51.08</v>
+        <v>50.26</v>
       </c>
     </row>
     <row r="75">
@@ -3726,7 +3726,7 @@
         <v>1</v>
       </c>
       <c r="I75" t="n">
-        <v>1.306</v>
+        <v>1.33</v>
       </c>
       <c r="J75" t="n">
         <v>128</v>
@@ -3735,7 +3735,7 @@
         <v>36</v>
       </c>
       <c r="L75" t="n">
-        <v>50.07</v>
+        <v>50.64</v>
       </c>
     </row>
     <row r="76">
@@ -3770,7 +3770,7 @@
         <v>1</v>
       </c>
       <c r="I76" t="n">
-        <v>1.172</v>
+        <v>1.311</v>
       </c>
       <c r="J76" t="n">
         <v>124</v>
@@ -3779,7 +3779,7 @@
         <v>30</v>
       </c>
       <c r="L76" t="n">
-        <v>50.42</v>
+        <v>50.78</v>
       </c>
     </row>
     <row r="77">
@@ -3814,7 +3814,7 @@
         <v>1</v>
       </c>
       <c r="I77" t="n">
-        <v>1.184</v>
+        <v>1.247</v>
       </c>
       <c r="J77" t="n">
         <v>125</v>
@@ -3823,7 +3823,7 @@
         <v>31</v>
       </c>
       <c r="L77" t="n">
-        <v>50.51</v>
+        <v>50.74</v>
       </c>
     </row>
     <row r="78">
@@ -3858,7 +3858,7 @@
         <v>1</v>
       </c>
       <c r="I78" t="n">
-        <v>1.231</v>
+        <v>1.247</v>
       </c>
       <c r="J78" t="n">
         <v>126</v>
@@ -3867,7 +3867,7 @@
         <v>33</v>
       </c>
       <c r="L78" t="n">
-        <v>50.28</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="79">
@@ -3902,7 +3902,7 @@
         <v>1</v>
       </c>
       <c r="I79" t="n">
-        <v>1.3</v>
+        <v>1.334</v>
       </c>
       <c r="J79" t="n">
         <v>128</v>
@@ -3911,7 +3911,7 @@
         <v>36</v>
       </c>
       <c r="L79" t="n">
-        <v>49.97</v>
+        <v>50.43</v>
       </c>
     </row>
     <row r="80">
@@ -3946,7 +3946,7 @@
         <v>1</v>
       </c>
       <c r="I80" t="n">
-        <v>1.142</v>
+        <v>1.188</v>
       </c>
       <c r="J80" t="n">
         <v>127</v>
@@ -3955,7 +3955,7 @@
         <v>29</v>
       </c>
       <c r="L80" t="n">
-        <v>50.86</v>
+        <v>51.36</v>
       </c>
     </row>
     <row r="81">
@@ -3990,7 +3990,7 @@
         <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>1.246</v>
+        <v>1.288</v>
       </c>
       <c r="J81" t="n">
         <v>127</v>
@@ -3999,7 +3999,7 @@
         <v>33</v>
       </c>
       <c r="L81" t="n">
-        <v>50.26</v>
+        <v>50.58</v>
       </c>
     </row>
     <row r="82">
@@ -4034,7 +4034,7 @@
         <v>1</v>
       </c>
       <c r="I82" t="n">
-        <v>1.289</v>
+        <v>1.344</v>
       </c>
       <c r="J82" t="n">
         <v>125</v>
@@ -4043,7 +4043,7 @@
         <v>35</v>
       </c>
       <c r="L82" t="n">
-        <v>49.19</v>
+        <v>48.74</v>
       </c>
     </row>
     <row r="83">
@@ -4078,7 +4078,7 @@
         <v>1</v>
       </c>
       <c r="I83" t="n">
-        <v>1.24</v>
+        <v>1.309</v>
       </c>
       <c r="J83" t="n">
         <v>126</v>
@@ -4087,7 +4087,7 @@
         <v>34</v>
       </c>
       <c r="L83" t="n">
-        <v>50.53</v>
+        <v>50.52</v>
       </c>
     </row>
     <row r="84">
@@ -4122,7 +4122,7 @@
         <v>1</v>
       </c>
       <c r="I84" t="n">
-        <v>1.312</v>
+        <v>1.342</v>
       </c>
       <c r="J84" t="n">
         <v>127</v>
@@ -4131,7 +4131,7 @@
         <v>35</v>
       </c>
       <c r="L84" t="n">
-        <v>48.72</v>
+        <v>48.89</v>
       </c>
     </row>
     <row r="85">
@@ -4166,7 +4166,7 @@
         <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>1.297</v>
+        <v>1.352</v>
       </c>
       <c r="J85" t="n">
         <v>127</v>
@@ -4175,7 +4175,7 @@
         <v>35</v>
       </c>
       <c r="L85" t="n">
-        <v>48.82</v>
+        <v>48.99</v>
       </c>
     </row>
     <row r="86">
@@ -4210,7 +4210,7 @@
         <v>1</v>
       </c>
       <c r="I86" t="n">
-        <v>1.15</v>
+        <v>1.182</v>
       </c>
       <c r="J86" t="n">
         <v>126</v>
@@ -4219,7 +4219,7 @@
         <v>29</v>
       </c>
       <c r="L86" t="n">
-        <v>50.58</v>
+        <v>51.61</v>
       </c>
     </row>
     <row r="87">
@@ -4254,7 +4254,7 @@
         <v>1</v>
       </c>
       <c r="I87" t="n">
-        <v>1.306</v>
+        <v>1.359</v>
       </c>
       <c r="J87" t="n">
         <v>127</v>
@@ -4263,7 +4263,7 @@
         <v>36</v>
       </c>
       <c r="L87" t="n">
-        <v>49.23</v>
+        <v>49.47</v>
       </c>
     </row>
     <row r="88">
@@ -4298,7 +4298,7 @@
         <v>1</v>
       </c>
       <c r="I88" t="n">
-        <v>1.333</v>
+        <v>1.407</v>
       </c>
       <c r="J88" t="n">
         <v>129</v>
@@ -4307,7 +4307,7 @@
         <v>37</v>
       </c>
       <c r="L88" t="n">
-        <v>49.15</v>
+        <v>49.1</v>
       </c>
     </row>
     <row r="89">
@@ -4342,7 +4342,7 @@
         <v>1</v>
       </c>
       <c r="I89" t="n">
-        <v>1.276</v>
+        <v>1.314</v>
       </c>
       <c r="J89" t="n">
         <v>128</v>
@@ -4351,7 +4351,7 @@
         <v>34</v>
       </c>
       <c r="L89" t="n">
-        <v>49.07</v>
+        <v>49.12</v>
       </c>
     </row>
     <row r="90">
@@ -4386,7 +4386,7 @@
         <v>1</v>
       </c>
       <c r="I90" t="n">
-        <v>1.415</v>
+        <v>1.435</v>
       </c>
       <c r="J90" t="n">
         <v>127</v>
@@ -4395,7 +4395,7 @@
         <v>41</v>
       </c>
       <c r="L90" t="n">
-        <v>48.93</v>
+        <v>49.04</v>
       </c>
     </row>
     <row r="91">
@@ -4430,7 +4430,7 @@
         <v>1</v>
       </c>
       <c r="I91" t="n">
-        <v>1.304</v>
+        <v>1.323</v>
       </c>
       <c r="J91" t="n">
         <v>127</v>
@@ -4439,7 +4439,7 @@
         <v>35</v>
       </c>
       <c r="L91" t="n">
-        <v>48.99</v>
+        <v>49.49</v>
       </c>
     </row>
     <row r="92">
@@ -4474,7 +4474,7 @@
         <v>1</v>
       </c>
       <c r="I92" t="n">
-        <v>1.232</v>
+        <v>1.277</v>
       </c>
       <c r="J92" t="n">
         <v>124</v>
@@ -4483,7 +4483,7 @@
         <v>33</v>
       </c>
       <c r="L92" t="n">
-        <v>50.49</v>
+        <v>50.59</v>
       </c>
     </row>
     <row r="93">
@@ -4518,7 +4518,7 @@
         <v>1</v>
       </c>
       <c r="I93" t="n">
-        <v>1.339</v>
+        <v>1.379</v>
       </c>
       <c r="J93" t="n">
         <v>126</v>
@@ -4527,7 +4527,7 @@
         <v>38</v>
       </c>
       <c r="L93" t="n">
-        <v>50.5</v>
+        <v>50.46</v>
       </c>
     </row>
     <row r="94">
@@ -4562,7 +4562,7 @@
         <v>1</v>
       </c>
       <c r="I94" t="n">
-        <v>1.341</v>
+        <v>1.382</v>
       </c>
       <c r="J94" t="n">
         <v>125</v>
@@ -4571,7 +4571,7 @@
         <v>38</v>
       </c>
       <c r="L94" t="n">
-        <v>50.31</v>
+        <v>50.19</v>
       </c>
     </row>
     <row r="95">
@@ -4606,7 +4606,7 @@
         <v>1</v>
       </c>
       <c r="I95" t="n">
-        <v>1.307</v>
+        <v>1.321</v>
       </c>
       <c r="J95" t="n">
         <v>128</v>
@@ -4615,7 +4615,7 @@
         <v>36</v>
       </c>
       <c r="L95" t="n">
-        <v>50.17</v>
+        <v>50.5</v>
       </c>
     </row>
     <row r="96">
@@ -4650,7 +4650,7 @@
         <v>1</v>
       </c>
       <c r="I96" t="n">
-        <v>1.169</v>
+        <v>1.213</v>
       </c>
       <c r="J96" t="n">
         <v>124</v>
@@ -4659,7 +4659,7 @@
         <v>29</v>
       </c>
       <c r="L96" t="n">
-        <v>49.43</v>
+        <v>49.38</v>
       </c>
     </row>
     <row r="97">
@@ -4694,7 +4694,7 @@
         <v>1</v>
       </c>
       <c r="I97" t="n">
-        <v>1.248</v>
+        <v>1.285</v>
       </c>
       <c r="J97" t="n">
         <v>124</v>
@@ -4703,7 +4703,7 @@
         <v>33</v>
       </c>
       <c r="L97" t="n">
-        <v>49.5</v>
+        <v>48.89</v>
       </c>
     </row>
     <row r="98">
@@ -4738,7 +4738,7 @@
         <v>1</v>
       </c>
       <c r="I98" t="n">
-        <v>1.403</v>
+        <v>1.418</v>
       </c>
       <c r="J98" t="n">
         <v>126</v>
@@ -4747,7 +4747,7 @@
         <v>40</v>
       </c>
       <c r="L98" t="n">
-        <v>49.93</v>
+        <v>50.32</v>
       </c>
     </row>
     <row r="99">
@@ -4782,7 +4782,7 @@
         <v>1</v>
       </c>
       <c r="I99" t="n">
-        <v>1.183</v>
+        <v>1.211</v>
       </c>
       <c r="J99" t="n">
         <v>129</v>
@@ -4791,7 +4791,7 @@
         <v>29</v>
       </c>
       <c r="L99" t="n">
-        <v>49.3</v>
+        <v>48.86</v>
       </c>
     </row>
     <row r="100">
@@ -4826,7 +4826,7 @@
         <v>1</v>
       </c>
       <c r="I100" t="n">
-        <v>1.301</v>
+        <v>1.353</v>
       </c>
       <c r="J100" t="n">
         <v>126</v>
@@ -4835,7 +4835,7 @@
         <v>36</v>
       </c>
       <c r="L100" t="n">
-        <v>50.48</v>
+        <v>50.05</v>
       </c>
     </row>
     <row r="101">
@@ -4870,7 +4870,7 @@
         <v>1</v>
       </c>
       <c r="I101" t="n">
-        <v>1.246</v>
+        <v>1.256</v>
       </c>
       <c r="J101" t="n">
         <v>127</v>
@@ -4879,7 +4879,7 @@
         <v>33</v>
       </c>
       <c r="L101" t="n">
-        <v>50.55</v>
+        <v>50.7</v>
       </c>
     </row>
     <row r="102">
@@ -4914,7 +4914,7 @@
         <v>1</v>
       </c>
       <c r="I102" t="n">
-        <v>1.236</v>
+        <v>1.268</v>
       </c>
       <c r="J102" t="n">
         <v>124</v>
@@ -4923,7 +4923,7 @@
         <v>33</v>
       </c>
       <c r="L102" t="n">
-        <v>50.51</v>
+        <v>50.56</v>
       </c>
     </row>
     <row r="103">
@@ -4958,7 +4958,7 @@
         <v>1</v>
       </c>
       <c r="I103" t="n">
-        <v>1.319</v>
+        <v>1.345</v>
       </c>
       <c r="J103" t="n">
         <v>123</v>
@@ -4967,7 +4967,7 @@
         <v>37</v>
       </c>
       <c r="L103" t="n">
-        <v>50.58</v>
+        <v>50.78</v>
       </c>
     </row>
     <row r="104">
@@ -5002,7 +5002,7 @@
         <v>1</v>
       </c>
       <c r="I104" t="n">
-        <v>1.241</v>
+        <v>1.259</v>
       </c>
       <c r="J104" t="n">
         <v>126</v>
@@ -5011,7 +5011,7 @@
         <v>33</v>
       </c>
       <c r="L104" t="n">
-        <v>50.79</v>
+        <v>50.63</v>
       </c>
     </row>
     <row r="105">
@@ -5046,7 +5046,7 @@
         <v>1</v>
       </c>
       <c r="I105" t="n">
-        <v>1.323</v>
+        <v>1.334</v>
       </c>
       <c r="J105" t="n">
         <v>128</v>
@@ -5055,7 +5055,7 @@
         <v>36</v>
       </c>
       <c r="L105" t="n">
-        <v>50.16</v>
+        <v>49.91</v>
       </c>
     </row>
     <row r="106">
@@ -5090,7 +5090,7 @@
         <v>1</v>
       </c>
       <c r="I106" t="n">
-        <v>1.215</v>
+        <v>1.214</v>
       </c>
       <c r="J106" t="n">
         <v>124</v>
@@ -5099,7 +5099,7 @@
         <v>30</v>
       </c>
       <c r="L106" t="n">
-        <v>50.63</v>
+        <v>50.87</v>
       </c>
     </row>
     <row r="107">
@@ -5134,7 +5134,7 @@
         <v>1</v>
       </c>
       <c r="I107" t="n">
-        <v>1.196</v>
+        <v>1.21</v>
       </c>
       <c r="J107" t="n">
         <v>125</v>
@@ -5143,7 +5143,7 @@
         <v>31</v>
       </c>
       <c r="L107" t="n">
-        <v>50.91</v>
+        <v>50.58</v>
       </c>
     </row>
     <row r="108">
@@ -5178,7 +5178,7 @@
         <v>1</v>
       </c>
       <c r="I108" t="n">
-        <v>1.244</v>
+        <v>1.296</v>
       </c>
       <c r="J108" t="n">
         <v>126</v>
@@ -5187,7 +5187,7 @@
         <v>33</v>
       </c>
       <c r="L108" t="n">
-        <v>50.5</v>
+        <v>50.02</v>
       </c>
     </row>
     <row r="109">
@@ -5222,7 +5222,7 @@
         <v>1</v>
       </c>
       <c r="I109" t="n">
-        <v>1.322</v>
+        <v>1.353</v>
       </c>
       <c r="J109" t="n">
         <v>128</v>
@@ -5231,7 +5231,7 @@
         <v>36</v>
       </c>
       <c r="L109" t="n">
-        <v>48.97</v>
+        <v>49.38</v>
       </c>
     </row>
     <row r="110">
@@ -5266,7 +5266,7 @@
         <v>1</v>
       </c>
       <c r="I110" t="n">
-        <v>1.168</v>
+        <v>1.201</v>
       </c>
       <c r="J110" t="n">
         <v>127</v>
@@ -5275,7 +5275,7 @@
         <v>29</v>
       </c>
       <c r="L110" t="n">
-        <v>50.53</v>
+        <v>50.78</v>
       </c>
     </row>
     <row r="111">
@@ -5310,7 +5310,7 @@
         <v>1</v>
       </c>
       <c r="I111" t="n">
-        <v>1.241</v>
+        <v>1.273</v>
       </c>
       <c r="J111" t="n">
         <v>127</v>
@@ -5319,7 +5319,7 @@
         <v>33</v>
       </c>
       <c r="L111" t="n">
-        <v>50.42</v>
+        <v>50.07</v>
       </c>
     </row>
     <row r="112">
@@ -5354,7 +5354,7 @@
         <v>1</v>
       </c>
       <c r="I112" t="n">
-        <v>1.313</v>
+        <v>1.347</v>
       </c>
       <c r="J112" t="n">
         <v>125</v>
@@ -5363,7 +5363,7 @@
         <v>35</v>
       </c>
       <c r="L112" t="n">
-        <v>49</v>
+        <v>49.16</v>
       </c>
     </row>
     <row r="113">
@@ -5398,7 +5398,7 @@
         <v>1</v>
       </c>
       <c r="I113" t="n">
-        <v>1.276</v>
+        <v>1.292</v>
       </c>
       <c r="J113" t="n">
         <v>126</v>
@@ -5407,7 +5407,7 @@
         <v>34</v>
       </c>
       <c r="L113" t="n">
-        <v>50.29</v>
+        <v>50.45</v>
       </c>
     </row>
     <row r="114">
@@ -5442,7 +5442,7 @@
         <v>1</v>
       </c>
       <c r="I114" t="n">
-        <v>1.311</v>
+        <v>1.335</v>
       </c>
       <c r="J114" t="n">
         <v>127</v>
@@ -5451,7 +5451,7 @@
         <v>35</v>
       </c>
       <c r="L114" t="n">
-        <v>49.16</v>
+        <v>48.82</v>
       </c>
     </row>
     <row r="115">
@@ -5486,7 +5486,7 @@
         <v>1</v>
       </c>
       <c r="I115" t="n">
-        <v>1.31</v>
+        <v>1.328</v>
       </c>
       <c r="J115" t="n">
         <v>127</v>
@@ -5495,7 +5495,7 @@
         <v>35</v>
       </c>
       <c r="L115" t="n">
-        <v>48.73</v>
+        <v>49.3</v>
       </c>
     </row>
     <row r="116">
@@ -5530,7 +5530,7 @@
         <v>1</v>
       </c>
       <c r="I116" t="n">
-        <v>1.165</v>
+        <v>1.21</v>
       </c>
       <c r="J116" t="n">
         <v>126</v>
@@ -5539,7 +5539,7 @@
         <v>29</v>
       </c>
       <c r="L116" t="n">
-        <v>50.43</v>
+        <v>50.67</v>
       </c>
     </row>
     <row r="117">
@@ -5574,7 +5574,7 @@
         <v>1</v>
       </c>
       <c r="I117" t="n">
-        <v>1.351</v>
+        <v>1.36</v>
       </c>
       <c r="J117" t="n">
         <v>127</v>
@@ -5583,7 +5583,7 @@
         <v>36</v>
       </c>
       <c r="L117" t="n">
-        <v>48.16</v>
+        <v>49.32</v>
       </c>
     </row>
     <row r="118">
@@ -5618,7 +5618,7 @@
         <v>1</v>
       </c>
       <c r="I118" t="n">
-        <v>1.353</v>
+        <v>1.389</v>
       </c>
       <c r="J118" t="n">
         <v>129</v>
@@ -5627,7 +5627,7 @@
         <v>37</v>
       </c>
       <c r="L118" t="n">
-        <v>49.3</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="119">
@@ -5662,7 +5662,7 @@
         <v>1</v>
       </c>
       <c r="I119" t="n">
-        <v>1.315</v>
+        <v>1.336</v>
       </c>
       <c r="J119" t="n">
         <v>128</v>
@@ -5671,7 +5671,7 @@
         <v>34</v>
       </c>
       <c r="L119" t="n">
-        <v>49.19</v>
+        <v>49.38</v>
       </c>
     </row>
     <row r="120">
@@ -5706,7 +5706,7 @@
         <v>1</v>
       </c>
       <c r="I120" t="n">
-        <v>1.44</v>
+        <v>1.472</v>
       </c>
       <c r="J120" t="n">
         <v>127</v>
@@ -5715,7 +5715,7 @@
         <v>41</v>
       </c>
       <c r="L120" t="n">
-        <v>48.94</v>
+        <v>48.93</v>
       </c>
     </row>
     <row r="121">
@@ -5750,7 +5750,7 @@
         <v>1</v>
       </c>
       <c r="I121" t="n">
-        <v>1.324</v>
+        <v>1.39</v>
       </c>
       <c r="J121" t="n">
         <v>127</v>
@@ -5759,7 +5759,7 @@
         <v>35</v>
       </c>
       <c r="L121" t="n">
-        <v>48.96</v>
+        <v>46.83</v>
       </c>
     </row>
   </sheetData>
@@ -6018,16 +6018,16 @@
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1.324</v>
+        <v>1.309</v>
       </c>
       <c r="I2" t="n">
-        <v>1.3</v>
+        <v>1.318</v>
       </c>
       <c r="J2" t="n">
-        <v>1.568</v>
+        <v>1.429</v>
       </c>
       <c r="K2" t="n">
-        <v>1.623</v>
+        <v>1.47</v>
       </c>
       <c r="L2" t="n">
         <v>126.2</v>
@@ -6144,7 +6144,7 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>1.431</v>
+        <v>1.308</v>
       </c>
       <c r="J2" t="n">
         <v>124</v>
@@ -6153,7 +6153,7 @@
         <v>33</v>
       </c>
       <c r="L2" t="n">
-        <v>38.32</v>
+        <v>48.11</v>
       </c>
     </row>
     <row r="3">
@@ -6188,7 +6188,7 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>1.461</v>
+        <v>1.232</v>
       </c>
       <c r="J3" t="n">
         <v>125</v>
@@ -6197,7 +6197,7 @@
         <v>31</v>
       </c>
       <c r="L3" t="n">
-        <v>38.59</v>
+        <v>50.31</v>
       </c>
     </row>
     <row r="4">
@@ -6232,7 +6232,7 @@
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>1.223</v>
+        <v>1.294</v>
       </c>
       <c r="J4" t="n">
         <v>124</v>
@@ -6241,7 +6241,7 @@
         <v>33</v>
       </c>
       <c r="L4" t="n">
-        <v>49.61</v>
+        <v>49.24</v>
       </c>
     </row>
     <row r="5">
@@ -6276,7 +6276,7 @@
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>1.171</v>
+        <v>1.222</v>
       </c>
       <c r="J5" t="n">
         <v>125</v>
@@ -6285,7 +6285,7 @@
         <v>31</v>
       </c>
       <c r="L5" t="n">
-        <v>50.68</v>
+        <v>50.36</v>
       </c>
     </row>
     <row r="6">
@@ -6320,7 +6320,7 @@
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>1.242</v>
+        <v>1.278</v>
       </c>
       <c r="J6" t="n">
         <v>124</v>
@@ -6329,7 +6329,7 @@
         <v>33</v>
       </c>
       <c r="L6" t="n">
-        <v>49.38</v>
+        <v>49.62</v>
       </c>
     </row>
     <row r="7">
@@ -6364,7 +6364,7 @@
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>1.184</v>
+        <v>1.247</v>
       </c>
       <c r="J7" t="n">
         <v>125</v>
@@ -6373,7 +6373,7 @@
         <v>31</v>
       </c>
       <c r="L7" t="n">
-        <v>50.51</v>
+        <v>50.74</v>
       </c>
     </row>
     <row r="8">
@@ -6408,7 +6408,7 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>1.248</v>
+        <v>1.285</v>
       </c>
       <c r="J8" t="n">
         <v>124</v>
@@ -6417,7 +6417,7 @@
         <v>33</v>
       </c>
       <c r="L8" t="n">
-        <v>49.5</v>
+        <v>48.89</v>
       </c>
     </row>
     <row r="9">
@@ -6452,7 +6452,7 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1.196</v>
+        <v>1.21</v>
       </c>
       <c r="J9" t="n">
         <v>125</v>
@@ -6461,7 +6461,7 @@
         <v>31</v>
       </c>
       <c r="L9" t="n">
-        <v>50.91</v>
+        <v>50.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>